<commit_message>
Add public schedule/emergency info page; QR opens it; check-in reads ?id=
</commit_message>
<xml_diff>
--- a/samples/sample_import.xlsx
+++ b/samples/sample_import.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4YNQ</t>
+          <t>5HJB</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HHJ3</t>
+          <t>B8HF</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>VAHA</t>
+          <t>ESH7</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PVFD</t>
+          <t>68Z4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>5PXN</t>
+          <t>9CNC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9NCP</t>
+          <t>62VX</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Y9GT</t>
+          <t>455Q</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>3DS8</t>
+          <t>VWYN</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>8BB3</t>
+          <t>EQ32</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>K4Y5</t>
+          <t>6CUK</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7NRA</t>
+          <t>LUH2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EKFB</t>
+          <t>C8PF</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">

</xml_diff>